<commit_message>
added a few of 3d printed helpers
</commit_message>
<xml_diff>
--- a/Robotic_Platform_v1/Orders/screws and washers/table of screws and washers.xlsx
+++ b/Robotic_Platform_v1/Orders/screws and washers/table of screws and washers.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\OSAMBot\Robotic_Platform_v1\Orders\screws + washers\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\OSAMBot\Robotic_Platform_v1\Orders\screws and washers\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E6DFF044-BEA2-434F-897D-80356F8AD70B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2545EB46-92A2-4740-AA02-C18F9469651F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="13905" xr2:uid="{6E515C7D-DDD6-4E98-BCCA-3CBC7FF96112}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>M6 zyl</t>
   </si>
@@ -108,6 +108,9 @@
       <t>length</t>
     </r>
   </si>
+  <si>
+    <t>slot nut M6</t>
+  </si>
 </sst>
 </file>
 
@@ -138,7 +141,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -154,6 +157,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="-0.249977111117893"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -212,7 +221,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -251,7 +260,16 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -568,17 +586,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D49B2A03-07F1-44AE-904C-148E3B8C1B07}">
-  <dimension ref="B2:AF47"/>
+  <dimension ref="B2:AG47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="14.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="4" bestFit="1" customWidth="1"/>
-    <col min="4" max="13" width="3" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.42578125" style="7"/>
+    <col min="4" max="4" width="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="3" customWidth="1"/>
+    <col min="6" max="14" width="3" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="11.42578125" style="7"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:32" ht="18.75" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:33" ht="18.75" x14ac:dyDescent="0.35">
       <c r="B2" s="21" t="s">
         <v>16</v>
       </c>
@@ -586,40 +606,42 @@
         <v>5</v>
       </c>
       <c r="D2" s="13">
+        <v>8</v>
+      </c>
+      <c r="E2" s="13">
         <v>10</v>
       </c>
-      <c r="E2" s="13">
+      <c r="F2" s="13">
         <v>15</v>
       </c>
-      <c r="F2" s="13">
+      <c r="G2" s="13">
         <v>16</v>
       </c>
-      <c r="G2" s="13">
+      <c r="H2" s="13">
         <v>20</v>
       </c>
-      <c r="H2" s="13">
+      <c r="I2" s="13">
         <v>25</v>
       </c>
-      <c r="I2" s="13">
+      <c r="J2" s="13">
         <v>30</v>
       </c>
-      <c r="J2" s="13">
+      <c r="K2" s="13">
         <v>35</v>
       </c>
-      <c r="K2" s="13">
+      <c r="L2" s="13">
         <v>40</v>
       </c>
-      <c r="L2" s="13">
+      <c r="M2" s="13">
         <v>50</v>
       </c>
-      <c r="M2" s="13">
+      <c r="N2" s="13">
         <v>60</v>
       </c>
-      <c r="N2" s="1"/>
       <c r="O2" s="1"/>
       <c r="P2" s="1"/>
-      <c r="Q2" s="8"/>
-      <c r="R2" s="1"/>
+      <c r="Q2" s="1"/>
+      <c r="R2" s="8"/>
       <c r="S2" s="1"/>
       <c r="T2" s="1"/>
       <c r="U2" s="1"/>
@@ -634,12 +656,13 @@
       <c r="AD2" s="1"/>
       <c r="AE2" s="1"/>
       <c r="AF2" s="1"/>
-    </row>
-    <row r="3" spans="2:32" x14ac:dyDescent="0.25">
+      <c r="AG2" s="1"/>
+    </row>
+    <row r="3" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B3" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="14">
+      <c r="C3" s="20">
         <v>12</v>
       </c>
       <c r="D3" s="14"/>
@@ -652,11 +675,11 @@
       <c r="K3" s="14"/>
       <c r="L3" s="14"/>
       <c r="M3" s="14"/>
-      <c r="N3" s="6"/>
+      <c r="N3" s="14"/>
       <c r="O3" s="6"/>
       <c r="P3" s="6"/>
-      <c r="Q3" s="9"/>
-      <c r="R3" s="6"/>
+      <c r="Q3" s="6"/>
+      <c r="R3" s="9"/>
       <c r="S3" s="6"/>
       <c r="T3" s="6"/>
       <c r="U3" s="6"/>
@@ -671,37 +694,37 @@
       <c r="AD3" s="6"/>
       <c r="AE3" s="6"/>
       <c r="AF3" s="6"/>
-    </row>
-    <row r="4" spans="2:32" x14ac:dyDescent="0.25">
+      <c r="AG3" s="6"/>
+    </row>
+    <row r="4" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B4" s="2" t="s">
         <v>1</v>
       </c>
       <c r="C4" s="15"/>
       <c r="D4" s="15"/>
-      <c r="E4" s="15">
+      <c r="E4" s="15"/>
+      <c r="G4" s="20">
         <v>16</v>
       </c>
-      <c r="F4" s="15"/>
-      <c r="G4" s="15"/>
-      <c r="H4" s="15">
+      <c r="H4" s="15"/>
+      <c r="I4" s="20">
         <v>16</v>
       </c>
-      <c r="I4" s="15">
+      <c r="J4" s="20">
         <v>16</v>
       </c>
-      <c r="J4" s="15"/>
-      <c r="K4" s="15">
+      <c r="K4" s="15"/>
+      <c r="L4" s="20">
         <v>16</v>
       </c>
-      <c r="L4" s="16">
+      <c r="M4" s="22">
         <v>16</v>
       </c>
-      <c r="M4" s="15"/>
-      <c r="N4" s="6"/>
+      <c r="N4" s="15"/>
       <c r="O4" s="6"/>
       <c r="P4" s="6"/>
-      <c r="Q4" s="9"/>
-      <c r="R4" s="6"/>
+      <c r="Q4" s="6"/>
+      <c r="R4" s="9"/>
       <c r="S4" s="6"/>
       <c r="T4" s="6"/>
       <c r="U4" s="6"/>
@@ -716,16 +739,17 @@
       <c r="AD4" s="6"/>
       <c r="AE4" s="6"/>
       <c r="AF4" s="6"/>
-    </row>
-    <row r="5" spans="2:32" x14ac:dyDescent="0.25">
+      <c r="AG4" s="6"/>
+    </row>
+    <row r="5" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B5" s="3" t="s">
         <v>5</v>
       </c>
       <c r="C5" s="14"/>
-      <c r="D5" s="14">
+      <c r="D5" s="20">
         <v>8</v>
       </c>
-      <c r="E5" s="14"/>
+      <c r="E5" s="16"/>
       <c r="F5" s="14"/>
       <c r="G5" s="14"/>
       <c r="H5" s="14"/>
@@ -734,11 +758,11 @@
       <c r="K5" s="14"/>
       <c r="L5" s="14"/>
       <c r="M5" s="14"/>
-      <c r="N5" s="6"/>
+      <c r="N5" s="14"/>
       <c r="O5" s="6"/>
       <c r="P5" s="6"/>
-      <c r="Q5" s="9"/>
-      <c r="R5" s="6"/>
+      <c r="Q5" s="6"/>
+      <c r="R5" s="9"/>
       <c r="S5" s="6"/>
       <c r="T5" s="6"/>
       <c r="U5" s="6"/>
@@ -753,34 +777,38 @@
       <c r="AD5" s="6"/>
       <c r="AE5" s="6"/>
       <c r="AF5" s="6"/>
-    </row>
-    <row r="6" spans="2:32" x14ac:dyDescent="0.25">
+      <c r="AG5" s="6"/>
+    </row>
+    <row r="6" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B6" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C6" s="15"/>
       <c r="D6" s="15"/>
       <c r="E6" s="15"/>
-      <c r="F6" s="15">
+      <c r="F6" s="15"/>
+      <c r="G6" s="20">
         <v>16</v>
       </c>
-      <c r="G6" s="15">
+      <c r="H6" s="20">
         <v>14</v>
       </c>
-      <c r="H6" s="15">
+      <c r="I6" s="20">
         <v>70</v>
       </c>
-      <c r="I6" s="17">
+      <c r="J6" s="23">
         <v>20</v>
       </c>
-      <c r="J6" s="17">
+      <c r="K6" s="23">
         <v>12</v>
       </c>
-      <c r="K6" s="17"/>
-      <c r="L6" s="17"/>
+      <c r="L6" s="23">
+        <v>12</v>
+      </c>
       <c r="M6" s="17"/>
-    </row>
-    <row r="7" spans="2:32" x14ac:dyDescent="0.25">
+      <c r="N6" s="17"/>
+    </row>
+    <row r="7" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B7" s="3" t="s">
         <v>12</v>
       </c>
@@ -790,37 +818,39 @@
       <c r="F7" s="14"/>
       <c r="G7" s="14"/>
       <c r="H7" s="14"/>
-      <c r="I7" s="18"/>
+      <c r="I7" s="14"/>
       <c r="J7" s="18"/>
-      <c r="K7" s="18">
+      <c r="K7" s="23">
         <v>12</v>
       </c>
       <c r="L7" s="18"/>
       <c r="M7" s="18"/>
-    </row>
-    <row r="8" spans="2:32" x14ac:dyDescent="0.25">
+      <c r="N7" s="18"/>
+    </row>
+    <row r="8" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B8" s="2" t="s">
         <v>2</v>
       </c>
       <c r="C8" s="15"/>
       <c r="D8" s="15"/>
       <c r="E8" s="15"/>
-      <c r="F8" s="15">
+      <c r="F8" s="15"/>
+      <c r="G8" s="20">
         <v>12</v>
       </c>
-      <c r="G8" s="15">
+      <c r="H8" s="20">
         <v>12</v>
       </c>
-      <c r="H8" s="15"/>
-      <c r="I8" s="17"/>
+      <c r="I8" s="15"/>
       <c r="J8" s="17"/>
-      <c r="K8" s="17">
+      <c r="K8" s="17"/>
+      <c r="L8" s="23">
         <v>32</v>
       </c>
-      <c r="L8" s="17"/>
       <c r="M8" s="17"/>
-    </row>
-    <row r="9" spans="2:32" x14ac:dyDescent="0.25">
+      <c r="N8" s="17"/>
+    </row>
+    <row r="9" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B9" s="3" t="s">
         <v>13</v>
       </c>
@@ -834,14 +864,14 @@
       <c r="J9" s="14"/>
       <c r="K9" s="14"/>
       <c r="L9" s="14"/>
-      <c r="M9" s="14">
+      <c r="M9" s="14"/>
+      <c r="N9" s="20">
         <v>16</v>
       </c>
-      <c r="N9" s="5"/>
       <c r="O9" s="5"/>
       <c r="P9" s="5"/>
-      <c r="Q9" s="10"/>
-      <c r="R9" s="5"/>
+      <c r="Q9" s="5"/>
+      <c r="R9" s="10"/>
       <c r="S9" s="5"/>
       <c r="T9" s="5"/>
       <c r="U9" s="5"/>
@@ -856,26 +886,30 @@
       <c r="AD9" s="5"/>
       <c r="AE9" s="5"/>
       <c r="AF9" s="5"/>
-    </row>
-    <row r="10" spans="2:32" x14ac:dyDescent="0.25">
+      <c r="AG9" s="5"/>
+    </row>
+    <row r="10" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B10" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C10" s="15"/>
       <c r="D10" s="15"/>
-      <c r="E10" s="15">
+      <c r="E10" s="20">
         <v>16</v>
       </c>
       <c r="F10" s="15"/>
-      <c r="G10" s="15"/>
+      <c r="G10" s="20">
+        <v>16</v>
+      </c>
       <c r="H10" s="15"/>
       <c r="I10" s="15"/>
       <c r="J10" s="15"/>
       <c r="K10" s="15"/>
       <c r="L10" s="15"/>
       <c r="M10" s="15"/>
-    </row>
-    <row r="11" spans="2:32" x14ac:dyDescent="0.25">
+      <c r="N10" s="15"/>
+    </row>
+    <row r="11" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B11" s="3" t="s">
         <v>14</v>
       </c>
@@ -885,15 +919,16 @@
       <c r="F11" s="14"/>
       <c r="G11" s="14"/>
       <c r="H11" s="14"/>
-      <c r="I11" s="20">
+      <c r="I11" s="14"/>
+      <c r="J11" s="20">
         <v>4</v>
       </c>
-      <c r="J11" s="14"/>
       <c r="K11" s="14"/>
       <c r="L11" s="14"/>
       <c r="M11" s="14"/>
-    </row>
-    <row r="12" spans="2:32" x14ac:dyDescent="0.25">
+      <c r="N11" s="14"/>
+    </row>
+    <row r="12" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B12" s="2" t="s">
         <v>15</v>
       </c>
@@ -901,19 +936,24 @@
       <c r="D12" s="15"/>
       <c r="E12" s="15"/>
       <c r="F12" s="15"/>
-      <c r="G12" s="20">
+      <c r="G12" s="15"/>
+      <c r="H12" s="20">
         <v>4</v>
       </c>
-      <c r="H12" s="15"/>
       <c r="I12" s="15"/>
       <c r="J12" s="15"/>
       <c r="K12" s="15"/>
       <c r="L12" s="15"/>
       <c r="M12" s="15"/>
-    </row>
-    <row r="13" spans="2:32" x14ac:dyDescent="0.25">
-      <c r="B13" s="12"/>
-      <c r="C13" s="19"/>
+      <c r="N12" s="15"/>
+    </row>
+    <row r="13" spans="2:33" x14ac:dyDescent="0.25">
+      <c r="B13" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="C13" s="25">
+        <v>8</v>
+      </c>
       <c r="D13" s="19"/>
       <c r="E13" s="19"/>
       <c r="F13" s="19"/>
@@ -924,11 +964,11 @@
       <c r="K13" s="19"/>
       <c r="L13" s="19"/>
       <c r="M13" s="19"/>
-      <c r="N13" s="4"/>
+      <c r="N13" s="19"/>
       <c r="O13" s="4"/>
       <c r="P13" s="4"/>
-      <c r="Q13" s="11"/>
-      <c r="R13" s="4"/>
+      <c r="Q13" s="4"/>
+      <c r="R13" s="11"/>
       <c r="S13" s="4"/>
       <c r="T13" s="4"/>
       <c r="U13" s="4"/>
@@ -943,13 +983,14 @@
       <c r="AD13" s="4"/>
       <c r="AE13" s="4"/>
       <c r="AF13" s="4"/>
-    </row>
-    <row r="14" spans="2:32" x14ac:dyDescent="0.25">
+      <c r="AG13" s="4"/>
+    </row>
+    <row r="14" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B14" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C14" s="22">
-        <f>Q21*2</f>
+      <c r="C14" s="24">
+        <f>R21*2</f>
         <v>160</v>
       </c>
       <c r="D14" s="15"/>
@@ -957,35 +998,36 @@
       <c r="F14" s="15"/>
       <c r="G14" s="15"/>
       <c r="H14" s="15"/>
-      <c r="I14" s="17"/>
+      <c r="I14" s="15"/>
       <c r="J14" s="17"/>
       <c r="K14" s="17"/>
       <c r="L14" s="17"/>
       <c r="M14" s="17"/>
-    </row>
-    <row r="15" spans="2:32" x14ac:dyDescent="0.25">
+      <c r="N14" s="17"/>
+    </row>
+    <row r="15" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B15" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C15" s="14">
-        <f>Q22*2</f>
-        <v>400</v>
+      <c r="C15" s="20">
+        <f>R22*2</f>
+        <v>424</v>
       </c>
       <c r="D15" s="14"/>
       <c r="E15" s="14"/>
       <c r="F15" s="14"/>
       <c r="G15" s="14"/>
       <c r="H15" s="14"/>
-      <c r="I15" s="18"/>
+      <c r="I15" s="14"/>
       <c r="J15" s="18"/>
       <c r="K15" s="18"/>
       <c r="L15" s="18"/>
       <c r="M15" s="18"/>
-      <c r="N15" s="4"/>
+      <c r="N15" s="18"/>
       <c r="O15" s="4"/>
       <c r="P15" s="4"/>
-      <c r="Q15" s="11"/>
-      <c r="R15" s="4"/>
+      <c r="Q15" s="4"/>
+      <c r="R15" s="11"/>
       <c r="S15" s="4"/>
       <c r="T15" s="4"/>
       <c r="U15" s="4"/>
@@ -1000,13 +1042,14 @@
       <c r="AD15" s="4"/>
       <c r="AE15" s="4"/>
       <c r="AF15" s="4"/>
-    </row>
-    <row r="16" spans="2:32" x14ac:dyDescent="0.25">
+      <c r="AG15" s="4"/>
+    </row>
+    <row r="16" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B16" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C16" s="15">
-        <f>Q23*2</f>
+      <c r="C16" s="20">
+        <f>R23*2</f>
         <v>32</v>
       </c>
       <c r="D16" s="15"/>
@@ -1014,13 +1057,14 @@
       <c r="F16" s="15"/>
       <c r="G16" s="15"/>
       <c r="H16" s="15"/>
-      <c r="I16" s="17"/>
+      <c r="I16" s="15"/>
       <c r="J16" s="17"/>
       <c r="K16" s="17"/>
       <c r="L16" s="17"/>
       <c r="M16" s="17"/>
-    </row>
-    <row r="17" spans="2:32" x14ac:dyDescent="0.25">
+      <c r="N16" s="17"/>
+    </row>
+    <row r="17" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B17" s="3"/>
       <c r="C17" s="5"/>
       <c r="D17" s="5"/>
@@ -1028,7 +1072,7 @@
       <c r="F17" s="5"/>
       <c r="G17" s="5"/>
       <c r="H17" s="5"/>
-      <c r="I17" s="4"/>
+      <c r="I17" s="5"/>
       <c r="J17" s="4"/>
       <c r="K17" s="4"/>
       <c r="L17" s="4"/>
@@ -1036,8 +1080,8 @@
       <c r="N17" s="4"/>
       <c r="O17" s="4"/>
       <c r="P17" s="4"/>
-      <c r="Q17" s="11"/>
-      <c r="R17" s="4"/>
+      <c r="Q17" s="4"/>
+      <c r="R17" s="11"/>
       <c r="S17" s="4"/>
       <c r="T17" s="4"/>
       <c r="U17" s="4"/>
@@ -1052,8 +1096,9 @@
       <c r="AD17" s="4"/>
       <c r="AE17" s="4"/>
       <c r="AF17" s="4"/>
-    </row>
-    <row r="18" spans="2:32" x14ac:dyDescent="0.25">
+      <c r="AG17" s="4"/>
+    </row>
+    <row r="18" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B18" s="2"/>
       <c r="C18" s="6"/>
       <c r="D18" s="6"/>
@@ -1061,8 +1106,9 @@
       <c r="F18" s="6"/>
       <c r="G18" s="6"/>
       <c r="H18" s="6"/>
-    </row>
-    <row r="19" spans="2:32" x14ac:dyDescent="0.25">
+      <c r="I18" s="6"/>
+    </row>
+    <row r="19" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B19" s="2"/>
       <c r="C19" s="6"/>
       <c r="D19" s="6"/>
@@ -1070,8 +1116,9 @@
       <c r="F19" s="6"/>
       <c r="G19" s="6"/>
       <c r="H19" s="6"/>
-    </row>
-    <row r="20" spans="2:32" x14ac:dyDescent="0.25">
+      <c r="I19" s="6"/>
+    </row>
+    <row r="20" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B20" s="2"/>
       <c r="C20" s="6"/>
       <c r="D20" s="6"/>
@@ -1079,8 +1126,9 @@
       <c r="F20" s="6"/>
       <c r="G20" s="6"/>
       <c r="H20" s="6"/>
-    </row>
-    <row r="21" spans="2:32" x14ac:dyDescent="0.25">
+      <c r="I20" s="6"/>
+    </row>
+    <row r="21" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B21" s="2"/>
       <c r="C21" s="6"/>
       <c r="D21" s="6"/>
@@ -1088,30 +1136,31 @@
       <c r="F21" s="6"/>
       <c r="G21" s="6"/>
       <c r="H21" s="6"/>
-      <c r="P21" s="6" t="s">
+      <c r="I21" s="6"/>
+      <c r="Q21" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="Q21" s="7">
-        <f>SUM(C4:M4)</f>
+      <c r="R21" s="7">
+        <f>SUM(C4:N4)</f>
         <v>80</v>
       </c>
     </row>
-    <row r="22" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B22" s="2"/>
       <c r="C22" s="6"/>
-      <c r="E22" s="6"/>
       <c r="F22" s="6"/>
       <c r="G22" s="6"/>
       <c r="H22" s="6"/>
-      <c r="P22" s="6" t="s">
+      <c r="I22" s="6"/>
+      <c r="Q22" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="Q22" s="7">
-        <f>SUM(C6:M8)</f>
-        <v>200</v>
-      </c>
-    </row>
-    <row r="23" spans="2:32" x14ac:dyDescent="0.25">
+      <c r="R22" s="7">
+        <f>SUM(C6:N8)</f>
+        <v>212</v>
+      </c>
+    </row>
+    <row r="23" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B23" s="2"/>
       <c r="C23" s="6"/>
       <c r="D23" s="6"/>
@@ -1119,15 +1168,16 @@
       <c r="F23" s="6"/>
       <c r="G23" s="6"/>
       <c r="H23" s="6"/>
-      <c r="P23" s="6" t="s">
+      <c r="I23" s="6"/>
+      <c r="Q23" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="Q23" s="7">
-        <f>SUM(C9:M9)</f>
+      <c r="R23" s="7">
+        <f>SUM(C9:N9)</f>
         <v>16</v>
       </c>
     </row>
-    <row r="24" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B24" s="2"/>
       <c r="C24" s="6"/>
       <c r="D24" s="6"/>
@@ -1135,8 +1185,9 @@
       <c r="F24" s="6"/>
       <c r="G24" s="6"/>
       <c r="H24" s="6"/>
-    </row>
-    <row r="25" spans="2:32" x14ac:dyDescent="0.25">
+      <c r="I24" s="6"/>
+    </row>
+    <row r="25" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B25" s="2"/>
       <c r="C25" s="6"/>
       <c r="D25" s="6"/>
@@ -1144,8 +1195,9 @@
       <c r="F25" s="6"/>
       <c r="G25" s="6"/>
       <c r="H25" s="6"/>
-    </row>
-    <row r="26" spans="2:32" x14ac:dyDescent="0.25">
+      <c r="I25" s="6"/>
+    </row>
+    <row r="26" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B26" s="2"/>
       <c r="C26" s="6"/>
       <c r="D26" s="6"/>
@@ -1153,8 +1205,9 @@
       <c r="F26" s="6"/>
       <c r="G26" s="6"/>
       <c r="H26" s="6"/>
-    </row>
-    <row r="27" spans="2:32" x14ac:dyDescent="0.25">
+      <c r="I26" s="6"/>
+    </row>
+    <row r="27" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B27" s="2"/>
       <c r="C27" s="6"/>
       <c r="D27" s="6"/>
@@ -1162,8 +1215,9 @@
       <c r="F27" s="6"/>
       <c r="G27" s="6"/>
       <c r="H27" s="6"/>
-    </row>
-    <row r="28" spans="2:32" x14ac:dyDescent="0.25">
+      <c r="I27" s="6"/>
+    </row>
+    <row r="28" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B28" s="2"/>
       <c r="C28" s="6"/>
       <c r="D28" s="6"/>
@@ -1171,8 +1225,9 @@
       <c r="F28" s="6"/>
       <c r="G28" s="6"/>
       <c r="H28" s="6"/>
-    </row>
-    <row r="29" spans="2:32" x14ac:dyDescent="0.25">
+      <c r="I28" s="6"/>
+    </row>
+    <row r="29" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B29" s="2"/>
       <c r="C29" s="6"/>
       <c r="D29" s="6"/>
@@ -1180,8 +1235,9 @@
       <c r="F29" s="6"/>
       <c r="G29" s="6"/>
       <c r="H29" s="6"/>
-    </row>
-    <row r="30" spans="2:32" x14ac:dyDescent="0.25">
+      <c r="I29" s="6"/>
+    </row>
+    <row r="30" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B30" s="2"/>
       <c r="C30" s="6"/>
       <c r="D30" s="6"/>
@@ -1189,8 +1245,9 @@
       <c r="F30" s="6"/>
       <c r="G30" s="6"/>
       <c r="H30" s="6"/>
-    </row>
-    <row r="31" spans="2:32" x14ac:dyDescent="0.25">
+      <c r="I30" s="6"/>
+    </row>
+    <row r="31" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B31" s="2"/>
       <c r="C31" s="6"/>
       <c r="D31" s="6"/>
@@ -1198,8 +1255,9 @@
       <c r="F31" s="6"/>
       <c r="G31" s="6"/>
       <c r="H31" s="6"/>
-    </row>
-    <row r="32" spans="2:32" x14ac:dyDescent="0.25">
+      <c r="I31" s="6"/>
+    </row>
+    <row r="32" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B32" s="2"/>
       <c r="C32" s="6"/>
       <c r="D32" s="6"/>
@@ -1207,8 +1265,9 @@
       <c r="F32" s="6"/>
       <c r="G32" s="6"/>
       <c r="H32" s="6"/>
-    </row>
-    <row r="33" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="I32" s="6"/>
+    </row>
+    <row r="33" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B33" s="2"/>
       <c r="C33" s="6"/>
       <c r="D33" s="6"/>
@@ -1216,8 +1275,9 @@
       <c r="F33" s="6"/>
       <c r="G33" s="6"/>
       <c r="H33" s="6"/>
-    </row>
-    <row r="34" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="I33" s="6"/>
+    </row>
+    <row r="34" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B34" s="2"/>
       <c r="C34" s="6"/>
       <c r="D34" s="6"/>
@@ -1225,8 +1285,9 @@
       <c r="F34" s="6"/>
       <c r="G34" s="6"/>
       <c r="H34" s="6"/>
-    </row>
-    <row r="35" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="I34" s="6"/>
+    </row>
+    <row r="35" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B35" s="2"/>
       <c r="C35" s="6"/>
       <c r="D35" s="6"/>
@@ -1234,8 +1295,9 @@
       <c r="F35" s="6"/>
       <c r="G35" s="6"/>
       <c r="H35" s="6"/>
-    </row>
-    <row r="36" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="I35" s="6"/>
+    </row>
+    <row r="36" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B36" s="2"/>
       <c r="C36" s="6"/>
       <c r="D36" s="6"/>
@@ -1243,8 +1305,9 @@
       <c r="F36" s="6"/>
       <c r="G36" s="6"/>
       <c r="H36" s="6"/>
-    </row>
-    <row r="37" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="I36" s="6"/>
+    </row>
+    <row r="37" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B37" s="2"/>
       <c r="C37" s="6"/>
       <c r="D37" s="6"/>
@@ -1252,8 +1315,9 @@
       <c r="F37" s="6"/>
       <c r="G37" s="6"/>
       <c r="H37" s="6"/>
-    </row>
-    <row r="38" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="I37" s="6"/>
+    </row>
+    <row r="38" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B38" s="2"/>
       <c r="C38" s="6"/>
       <c r="D38" s="6"/>
@@ -1261,8 +1325,9 @@
       <c r="F38" s="6"/>
       <c r="G38" s="6"/>
       <c r="H38" s="6"/>
-    </row>
-    <row r="39" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="I38" s="6"/>
+    </row>
+    <row r="39" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B39" s="2"/>
       <c r="C39" s="6"/>
       <c r="D39" s="6"/>
@@ -1270,8 +1335,9 @@
       <c r="F39" s="6"/>
       <c r="G39" s="6"/>
       <c r="H39" s="6"/>
-    </row>
-    <row r="40" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="I39" s="6"/>
+    </row>
+    <row r="40" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B40" s="2"/>
       <c r="C40" s="6"/>
       <c r="D40" s="6"/>
@@ -1279,8 +1345,9 @@
       <c r="F40" s="6"/>
       <c r="G40" s="6"/>
       <c r="H40" s="6"/>
-    </row>
-    <row r="41" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="I40" s="6"/>
+    </row>
+    <row r="41" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B41" s="2"/>
       <c r="C41" s="6"/>
       <c r="D41" s="6"/>
@@ -1288,8 +1355,9 @@
       <c r="F41" s="6"/>
       <c r="G41" s="6"/>
       <c r="H41" s="6"/>
-    </row>
-    <row r="42" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="I41" s="6"/>
+    </row>
+    <row r="42" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B42" s="2"/>
       <c r="C42" s="6"/>
       <c r="D42" s="6"/>
@@ -1297,8 +1365,9 @@
       <c r="F42" s="6"/>
       <c r="G42" s="6"/>
       <c r="H42" s="6"/>
-    </row>
-    <row r="43" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="I42" s="6"/>
+    </row>
+    <row r="43" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B43" s="2"/>
       <c r="C43" s="6"/>
       <c r="D43" s="6"/>
@@ -1306,8 +1375,9 @@
       <c r="F43" s="6"/>
       <c r="G43" s="6"/>
       <c r="H43" s="6"/>
-    </row>
-    <row r="44" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="I43" s="6"/>
+    </row>
+    <row r="44" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B44" s="2"/>
       <c r="C44" s="6"/>
       <c r="D44" s="6"/>
@@ -1315,8 +1385,9 @@
       <c r="F44" s="6"/>
       <c r="G44" s="6"/>
       <c r="H44" s="6"/>
-    </row>
-    <row r="45" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="I44" s="6"/>
+    </row>
+    <row r="45" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B45" s="2"/>
       <c r="C45" s="6"/>
       <c r="D45" s="6"/>
@@ -1324,8 +1395,9 @@
       <c r="F45" s="6"/>
       <c r="G45" s="6"/>
       <c r="H45" s="6"/>
-    </row>
-    <row r="46" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="I45" s="6"/>
+    </row>
+    <row r="46" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B46" s="2"/>
       <c r="C46" s="6"/>
       <c r="D46" s="6"/>
@@ -1333,8 +1405,9 @@
       <c r="F46" s="6"/>
       <c r="G46" s="6"/>
       <c r="H46" s="6"/>
-    </row>
-    <row r="47" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="I46" s="6"/>
+    </row>
+    <row r="47" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B47" s="2"/>
       <c r="C47" s="6"/>
       <c r="D47" s="6"/>
@@ -1342,6 +1415,7 @@
       <c r="F47" s="6"/>
       <c r="G47" s="6"/>
       <c r="H47" s="6"/>
+      <c r="I47" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>

</xml_diff>